<commit_message>
Fix assessment import to accept reference number and commit template file for Render deployment
- Update ExcelBulkImporter to auto-detect headers and support both 'Student Number' and 'Reference Number' columns
- Fix import_excel route to lookup students by either student_number or reference_number
- Add regression test for reference number header detection
- Commit student_template.xlsx to ensure template availability on Render
- Add lxml to requirements.txt for template XML operations
</commit_message>
<xml_diff>
--- a/templates_excel/student_template.xlsx
+++ b/templates_excel/student_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\school_assess_app_EXPERIMENTAL\templates_excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\school_assess_app_EXPERIMENTAL_ver_1\templates_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F373997-99C6-449F-BC06-08FEC4AF01C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3624DEE-B2C8-457D-A6B9-1EE27CCB4A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="89">
   <si>
     <t>SCHOOL:</t>
   </si>
@@ -70,12 +70,6 @@
     <t>PRACTICAL PORTFOLIO</t>
   </si>
   <si>
-    <t>MID TERM EXAMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> TOTAL CLASS SCORE</t>
-  </si>
-  <si>
     <t>100% OF TOTAL CLASS SCORE</t>
   </si>
   <si>
@@ -97,16 +91,7 @@
     <t>Points/Weighting:</t>
   </si>
   <si>
-    <t>Serial Number</t>
-  </si>
-  <si>
     <t>Name of Students</t>
-  </si>
-  <si>
-    <t>Ref. Id</t>
-  </si>
-  <si>
-    <t>Study Area</t>
   </si>
   <si>
     <t>%</t>
@@ -261,6 +246,48 @@
   <si>
     <t>[42]</t>
   </si>
+  <si>
+    <t>Student Number</t>
+  </si>
+  <si>
+    <t>Reference Number</t>
+  </si>
+  <si>
+    <t>Learning Area</t>
+  </si>
+  <si>
+    <t>Mid-Semester Exam</t>
+  </si>
+  <si>
+    <t>Total Class Score</t>
+  </si>
+  <si>
+    <t>ica1</t>
+  </si>
+  <si>
+    <t>ica2</t>
+  </si>
+  <si>
+    <t>icp1</t>
+  </si>
+  <si>
+    <t>icp2</t>
+  </si>
+  <si>
+    <t>gp1</t>
+  </si>
+  <si>
+    <t>gp2</t>
+  </si>
+  <si>
+    <t>practical</t>
+  </si>
+  <si>
+    <t>mid_term</t>
+  </si>
+  <si>
+    <t>end_term</t>
+  </si>
 </sst>
 </file>
 
@@ -274,7 +301,7 @@
     <numFmt numFmtId="167" formatCode="General;;&quot;&quot;;@"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="47" x14ac:knownFonts="1">
+  <fonts count="48" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -575,6 +602,12 @@
       <sz val="9"/>
       <name val="Comic Sans MS"/>
       <family val="4"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="16">
@@ -918,7 +951,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
@@ -1327,10 +1360,13 @@
     <xf numFmtId="0" fontId="45" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="47" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="41" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1990,24 +2026,24 @@
       <c r="U5" s="14"/>
     </row>
     <row r="6" spans="1:31" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="112" t="s">
+      <c r="E6" s="113" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="111"/>
+      <c r="F6" s="112"/>
       <c r="G6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="110" t="s">
+      <c r="H6" s="111" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="111"/>
+      <c r="I6" s="112"/>
       <c r="J6" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="K6" s="110" t="s">
+      <c r="K6" s="111" t="s">
         <v>13</v>
       </c>
-      <c r="L6" s="111"/>
+      <c r="L6" s="112"/>
       <c r="M6" s="15" t="s">
         <v>14</v>
       </c>
@@ -2015,38 +2051,38 @@
         <v>15</v>
       </c>
       <c r="O6" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="P6" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q6" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="P6" s="17" t="s">
+      <c r="R6" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="Q6" s="18" t="s">
+      <c r="S6" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="R6" s="19" t="s">
+      <c r="T6" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="S6" s="20" t="s">
+      <c r="U6" s="21" t="s">
         <v>20</v>
-      </c>
-      <c r="T6" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="U6" s="21" t="s">
-        <v>22</v>
       </c>
       <c r="W6" s="22"/>
     </row>
     <row r="7" spans="1:31" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C7" s="24">
         <f>COUNTA(B10:B110)</f>
         <v>0</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E7" s="26">
         <v>50</v>
@@ -2128,47 +2164,65 @@
       <c r="W8" s="32"/>
       <c r="X8" s="33"/>
     </row>
-    <row r="9" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="107" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="B9" s="108" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="109" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
+        <v>23</v>
+      </c>
+      <c r="C9" s="109" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" s="110" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="F9" s="36" t="s">
+        <v>81</v>
+      </c>
       <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
+      <c r="H9" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="I9" s="36" t="s">
+        <v>83</v>
+      </c>
       <c r="J9" s="36"/>
-      <c r="K9" s="36"/>
-      <c r="L9" s="36"/>
+      <c r="K9" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="L9" s="36" t="s">
+        <v>85</v>
+      </c>
       <c r="M9" s="36"/>
-      <c r="N9" s="36"/>
-      <c r="O9" s="36"/>
+      <c r="N9" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="O9" s="36" t="s">
+        <v>87</v>
+      </c>
       <c r="P9" s="36"/>
       <c r="Q9" s="36"/>
       <c r="R9" s="37"/>
-      <c r="S9" s="36"/>
+      <c r="S9" s="36" t="s">
+        <v>88</v>
+      </c>
       <c r="T9" s="37"/>
       <c r="U9" s="38"/>
       <c r="V9" s="39" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="W9" s="39" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="X9" s="39" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="Z9" s="40" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
@@ -2329,7 +2383,7 @@
         <v>F9</v>
       </c>
       <c r="Z11" s="56" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
@@ -2411,7 +2465,7 @@
         <v>F9</v>
       </c>
       <c r="Z12" s="56" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
@@ -2493,7 +2547,7 @@
         <v>F9</v>
       </c>
       <c r="Z13" s="56" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
@@ -2575,7 +2629,7 @@
         <v>F9</v>
       </c>
       <c r="Z14" s="56" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
@@ -2657,7 +2711,7 @@
         <v>F9</v>
       </c>
       <c r="Z15" s="56" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
@@ -2739,7 +2793,7 @@
         <v>F9</v>
       </c>
       <c r="Z16" s="56" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.25">
@@ -2821,7 +2875,7 @@
         <v>F9</v>
       </c>
       <c r="Z17" s="56" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.25">
@@ -2903,7 +2957,7 @@
         <v>F9</v>
       </c>
       <c r="Z18" s="56" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.25">
@@ -2985,7 +3039,7 @@
         <v>F9</v>
       </c>
       <c r="Z19" s="56" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.25">
@@ -3067,7 +3121,7 @@
         <v>F9</v>
       </c>
       <c r="Z20" s="56" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:29" x14ac:dyDescent="0.25">
@@ -3229,10 +3283,10 @@
         <v>F9</v>
       </c>
       <c r="Z22" s="57" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="AA22" s="58" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:29" x14ac:dyDescent="0.25">
@@ -3393,7 +3447,7 @@
         <v>F9</v>
       </c>
       <c r="Z24" s="59" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="AA24" s="60" t="b">
         <v>0</v>
@@ -3636,16 +3690,16 @@
         <v>F9</v>
       </c>
       <c r="Z27" s="61" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="AA27" s="61" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="AB27" s="62" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="AC27" s="61" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.25">
@@ -3727,13 +3781,13 @@
         <v>F9</v>
       </c>
       <c r="Z28" s="63" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="AA28" s="64" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="AB28" s="65" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="AC28" s="66">
         <v>4</v>
@@ -3818,13 +3872,13 @@
         <v>F9</v>
       </c>
       <c r="Z29" s="63" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="AA29" s="64" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="AB29" s="65" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="AC29" s="66">
         <v>3.5</v>
@@ -3909,13 +3963,13 @@
         <v>F9</v>
       </c>
       <c r="Z30" s="63" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="AA30" s="64" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="AB30" s="65" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="AC30" s="66">
         <v>3</v>
@@ -4000,13 +4054,13 @@
         <v>F9</v>
       </c>
       <c r="Z31" s="63" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="AA31" s="64" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AB31" s="65" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="AC31" s="66">
         <v>2.5</v>
@@ -4091,13 +4145,13 @@
         <v>F9</v>
       </c>
       <c r="Z32" s="63" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="AA32" s="64" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="AB32" s="65" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="AC32" s="66">
         <v>2</v>
@@ -4182,13 +4236,13 @@
         <v>F9</v>
       </c>
       <c r="Z33" s="63" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="AA33" s="64" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="AB33" s="65" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="AC33" s="66">
         <v>1.5</v>
@@ -4273,13 +4327,13 @@
         <v>F9</v>
       </c>
       <c r="Z34" s="63" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="AA34" s="64" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="AB34" s="65" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="AC34" s="66">
         <v>1</v>
@@ -4364,13 +4418,13 @@
         <v>F9</v>
       </c>
       <c r="Z35" s="63" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="AA35" s="64" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="AB35" s="65" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="AC35" s="66">
         <v>0.5</v>
@@ -4455,13 +4509,13 @@
         <v>F9</v>
       </c>
       <c r="Z36" s="63" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="AA36" s="64" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="AB36" s="65" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="AC36" s="66">
         <v>0</v>
@@ -4703,10 +4757,10 @@
         <f t="shared" si="10"/>
         <v>F9</v>
       </c>
-      <c r="Z39" s="113" t="s">
-        <v>73</v>
-      </c>
-      <c r="AA39" s="114"/>
+      <c r="Z39" s="114" t="s">
+        <v>68</v>
+      </c>
+      <c r="AA39" s="115"/>
     </row>
     <row r="40" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="41">
@@ -4787,10 +4841,10 @@
         <v>F9</v>
       </c>
       <c r="Z40" s="67" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="AA40" s="68" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:30" x14ac:dyDescent="0.25">
@@ -4872,7 +4926,7 @@
         <v>F9</v>
       </c>
       <c r="Z41" s="69" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="AA41" s="70">
         <f>COUNTIF(X$7:$X86,"a1")</f>
@@ -4958,7 +5012,7 @@
         <v>F9</v>
       </c>
       <c r="Z42" s="69" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="AA42" s="70">
         <f>COUNTIF(X$7:$X262,"B2")</f>
@@ -5044,7 +5098,7 @@
         <v>F9</v>
       </c>
       <c r="Z43" s="69" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="AA43" s="70">
         <f>COUNTIF(X$7:$X263,"b3")</f>
@@ -5130,7 +5184,7 @@
         <v>F9</v>
       </c>
       <c r="Z44" s="69" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="AA44" s="70">
         <f>COUNTIF(X$7:$X264,"c4")</f>
@@ -5216,7 +5270,7 @@
         <v>F9</v>
       </c>
       <c r="Z45" s="69" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="AA45" s="70">
         <f>COUNTIF(X$7:$X265,"c5")</f>
@@ -5305,7 +5359,7 @@
         <v>F9</v>
       </c>
       <c r="Z46" s="69" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="AA46" s="70">
         <f>COUNTIF(X$7:$X266,"c6")</f>
@@ -5394,7 +5448,7 @@
         <v>F9</v>
       </c>
       <c r="Z47" s="69" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="AA47" s="70">
         <f>COUNTIF(X$7:$X267,"d7")</f>
@@ -5483,7 +5537,7 @@
         <v>F9</v>
       </c>
       <c r="Z48" s="69" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="AA48" s="70">
         <f>COUNTIF(X$7:$X268,"e8")</f>
@@ -5572,7 +5626,7 @@
         <v>F9</v>
       </c>
       <c r="Z49" s="73" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="AA49" s="74">
         <f>COUNTIF(X10:X71,"f9")</f>
@@ -5661,7 +5715,7 @@
         <v>F9</v>
       </c>
       <c r="Z50" s="75" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="AA50" s="76">
         <f>SUM(AA41:AA49)</f>
@@ -11768,7 +11822,7 @@
     <row r="126" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A126" s="96"/>
       <c r="B126" s="97" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C126" s="97"/>
       <c r="D126" s="97"/>
@@ -11805,7 +11859,7 @@
     <row r="127" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A127" s="96"/>
       <c r="B127" s="97" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C127" s="97"/>
       <c r="D127" s="97"/>
@@ -11839,7 +11893,7 @@
     <row r="128" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A128" s="96"/>
       <c r="B128" s="97" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C128" s="97"/>
       <c r="D128" s="97"/>
@@ -11865,7 +11919,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="X128" s="103" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>